<commit_message>
Implementar requisiciones y flujo de entrega desde almacén
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/storage/templates/tarjetas_responsabilidad.xlsx
+++ b/storage/templates/tarjetas_responsabilidad.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\sistema_hospital\storage\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8D35F48-95F6-4399-94BE-BF6FD8DD5685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA4921A-77F7-478E-878E-CC1B891AC412}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="881" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -210,7 +210,7 @@
     <numFmt numFmtId="166" formatCode="&quot;Q&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="_-[$Q-100A]* #,##0.00_-;\-[$Q-100A]* #,##0.00_-;_-[$Q-100A]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -304,6 +304,17 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -341,7 +352,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -388,14 +399,8 @@
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -403,20 +408,11 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="2" borderId="0" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
@@ -426,9 +422,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -483,26 +476,104 @@
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="2" borderId="0" xfId="6" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="5" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="17" fillId="0" borderId="0" xfId="10" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -822,15 +893,15 @@
     <row r="4" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="55" t="s">
+      <c r="C4" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="56" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="56"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="47"/>
       <c r="I4" s="7"/>
     </row>
     <row r="5" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.35">
@@ -847,15 +918,15 @@
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56" t="s">
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="56"/>
+      <c r="G6" s="47"/>
     </row>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
@@ -885,530 +956,530 @@
       <c r="D10" s="15"/>
       <c r="E10" s="16"/>
     </row>
-    <row r="11" spans="1:9" s="22" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="17">
+    <row r="11" spans="1:9" s="20" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="53">
         <v>38717</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="19">
-        <v>1</v>
-      </c>
-      <c r="D11" s="20" t="s">
+      <c r="C11" s="55">
+        <v>1</v>
+      </c>
+      <c r="D11" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="44">
+      <c r="E11" s="56">
         <v>125</v>
       </c>
-      <c r="F11" s="45"/>
-      <c r="G11" s="46">
+      <c r="F11" s="57"/>
+      <c r="G11" s="58">
         <f>(E11)</f>
         <v>125</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="22" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17">
+    <row r="12" spans="1:9" s="20" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="53">
         <v>45127</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="24">
-        <v>1</v>
-      </c>
-      <c r="D12" s="20" t="s">
+      <c r="C12" s="60">
+        <v>1</v>
+      </c>
+      <c r="D12" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="44">
+      <c r="E12" s="56">
         <v>949</v>
       </c>
-      <c r="F12" s="47"/>
-      <c r="G12" s="46">
+      <c r="F12" s="61"/>
+      <c r="G12" s="58">
         <f t="shared" ref="G12:G31" si="0">G11+E12</f>
         <v>1074</v>
       </c>
     </row>
-    <row r="13" spans="1:9" s="28" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="17">
+    <row r="13" spans="1:9" s="23" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="53">
         <v>41506</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="26">
-        <v>1</v>
-      </c>
-      <c r="D13" s="27" t="s">
+      <c r="C13" s="63">
+        <v>1</v>
+      </c>
+      <c r="D13" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="47">
+      <c r="E13" s="61">
         <v>334</v>
       </c>
-      <c r="F13" s="46"/>
-      <c r="G13" s="46">
+      <c r="F13" s="58"/>
+      <c r="G13" s="58">
         <f t="shared" si="0"/>
         <v>1408</v>
       </c>
     </row>
-    <row r="14" spans="1:9" s="28" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B14" s="29" t="s">
+    <row r="14" spans="1:9" s="23" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B14" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="29">
-        <v>1</v>
-      </c>
-      <c r="D14" s="30" t="s">
+      <c r="C14" s="64">
+        <v>1</v>
+      </c>
+      <c r="D14" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46">
+      <c r="E14" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58">
         <f t="shared" si="0"/>
         <v>17908</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B15" s="26" t="s">
+      <c r="A15" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B15" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="29">
-        <v>1</v>
-      </c>
-      <c r="D15" s="30" t="s">
+      <c r="C15" s="64">
+        <v>1</v>
+      </c>
+      <c r="D15" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="E15" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46">
+      <c r="E15" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58">
         <f t="shared" si="0"/>
         <v>34408</v>
       </c>
-      <c r="H15" s="31"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="1:9" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B16" s="29" t="s">
+      <c r="A16" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B16" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="29">
-        <v>1</v>
-      </c>
-      <c r="D16" s="30" t="s">
+      <c r="C16" s="64">
+        <v>1</v>
+      </c>
+      <c r="D16" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F16" s="46"/>
-      <c r="G16" s="46">
+      <c r="E16" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F16" s="58"/>
+      <c r="G16" s="58">
         <f t="shared" si="0"/>
         <v>50908</v>
       </c>
-      <c r="H16" s="31"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B17" s="26" t="s">
+      <c r="A17" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B17" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="26">
-        <v>1</v>
-      </c>
-      <c r="D17" s="30" t="s">
+      <c r="C17" s="63">
+        <v>1</v>
+      </c>
+      <c r="D17" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46">
+      <c r="E17" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58">
         <f t="shared" si="0"/>
         <v>67408</v>
       </c>
-      <c r="H17" s="31"/>
+      <c r="H17" s="26"/>
     </row>
     <row r="18" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B18" s="26" t="s">
+      <c r="A18" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B18" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="26">
-        <v>1</v>
-      </c>
-      <c r="D18" s="30" t="s">
+      <c r="C18" s="63">
+        <v>1</v>
+      </c>
+      <c r="D18" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46">
+      <c r="E18" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58">
         <f t="shared" si="0"/>
         <v>83908</v>
       </c>
-      <c r="H18" s="31"/>
+      <c r="H18" s="26"/>
     </row>
     <row r="19" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B19" s="32" t="s">
+      <c r="A19" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B19" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="29">
-        <v>1</v>
-      </c>
-      <c r="D19" s="30" t="s">
+      <c r="C19" s="64">
+        <v>1</v>
+      </c>
+      <c r="D19" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F19" s="46"/>
-      <c r="G19" s="46">
+      <c r="E19" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F19" s="58"/>
+      <c r="G19" s="58">
         <f t="shared" si="0"/>
         <v>100408</v>
       </c>
-      <c r="H19" s="31"/>
+      <c r="H19" s="26"/>
     </row>
     <row r="20" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B20" s="26" t="s">
+      <c r="A20" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B20" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="26">
-        <v>1</v>
-      </c>
-      <c r="D20" s="30" t="s">
+      <c r="C20" s="63">
+        <v>1</v>
+      </c>
+      <c r="D20" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46">
+      <c r="E20" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F20" s="58"/>
+      <c r="G20" s="58">
         <f t="shared" si="0"/>
         <v>116908</v>
       </c>
-      <c r="H20" s="31"/>
+      <c r="H20" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B21" s="26" t="s">
+      <c r="A21" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B21" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="26">
-        <v>1</v>
-      </c>
-      <c r="D21" s="30" t="s">
+      <c r="C21" s="63">
+        <v>1</v>
+      </c>
+      <c r="D21" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F21" s="46"/>
-      <c r="G21" s="46">
+      <c r="E21" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F21" s="58"/>
+      <c r="G21" s="58">
         <f t="shared" si="0"/>
         <v>133408</v>
       </c>
-      <c r="H21" s="31"/>
+      <c r="H21" s="26"/>
     </row>
     <row r="22" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B22" s="29" t="s">
+      <c r="A22" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B22" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="29">
-        <v>1</v>
-      </c>
-      <c r="D22" s="30" t="s">
+      <c r="C22" s="64">
+        <v>1</v>
+      </c>
+      <c r="D22" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F22" s="46"/>
-      <c r="G22" s="46">
+      <c r="E22" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58">
         <f t="shared" si="0"/>
         <v>149908</v>
       </c>
-      <c r="H22" s="31"/>
+      <c r="H22" s="26"/>
     </row>
     <row r="23" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B23" s="33" t="s">
+      <c r="A23" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B23" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="29">
-        <v>1</v>
-      </c>
-      <c r="D23" s="30" t="s">
+      <c r="C23" s="64">
+        <v>1</v>
+      </c>
+      <c r="D23" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="47">
-        <v>16500</v>
-      </c>
-      <c r="F23" s="45"/>
-      <c r="G23" s="46">
+      <c r="E23" s="61">
+        <v>16500</v>
+      </c>
+      <c r="F23" s="57"/>
+      <c r="G23" s="58">
         <f t="shared" si="0"/>
         <v>166408</v>
       </c>
-      <c r="H23" s="31"/>
-    </row>
-    <row r="24" spans="1:8" s="35" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B24" s="25" t="s">
+      <c r="H23" s="26"/>
+    </row>
+    <row r="24" spans="1:8" s="29" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B24" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="29">
-        <v>1</v>
-      </c>
-      <c r="D24" s="30" t="s">
+      <c r="C24" s="64">
+        <v>1</v>
+      </c>
+      <c r="D24" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F24" s="45"/>
-      <c r="G24" s="46">
+      <c r="E24" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F24" s="57"/>
+      <c r="G24" s="58">
         <f t="shared" si="0"/>
         <v>182908</v>
       </c>
-      <c r="H24" s="34"/>
-    </row>
-    <row r="25" spans="1:8" s="35" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B25" s="29" t="s">
+      <c r="H24" s="28"/>
+    </row>
+    <row r="25" spans="1:8" s="29" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B25" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="29">
-        <v>1</v>
-      </c>
-      <c r="D25" s="30" t="s">
+      <c r="C25" s="64">
+        <v>1</v>
+      </c>
+      <c r="D25" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="E25" s="47">
-        <v>16500</v>
-      </c>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46">
+      <c r="E25" s="61">
+        <v>16500</v>
+      </c>
+      <c r="F25" s="58"/>
+      <c r="G25" s="58">
         <f t="shared" si="0"/>
         <v>199408</v>
       </c>
-      <c r="H25" s="34"/>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B26" s="25" t="s">
+      <c r="A26" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B26" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="29">
-        <v>1</v>
-      </c>
-      <c r="D26" s="30" t="s">
+      <c r="C26" s="64">
+        <v>1</v>
+      </c>
+      <c r="D26" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="E26" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F26" s="46"/>
-      <c r="G26" s="46">
+      <c r="E26" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58">
         <f t="shared" si="0"/>
         <v>215908</v>
       </c>
-      <c r="H26" s="31"/>
+      <c r="H26" s="26"/>
     </row>
     <row r="27" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B27" s="25" t="s">
+      <c r="A27" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B27" s="62" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="29">
-        <v>1</v>
-      </c>
-      <c r="D27" s="30" t="s">
+      <c r="C27" s="64">
+        <v>1</v>
+      </c>
+      <c r="D27" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="47">
-        <v>16500</v>
-      </c>
-      <c r="F27" s="46"/>
-      <c r="G27" s="46">
+      <c r="E27" s="61">
+        <v>16500</v>
+      </c>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58">
         <f t="shared" si="0"/>
         <v>232408</v>
       </c>
-      <c r="H27" s="31"/>
+      <c r="H27" s="26"/>
     </row>
     <row r="28" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B28" s="26" t="s">
+      <c r="A28" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B28" s="63" t="s">
         <v>43</v>
       </c>
-      <c r="C28" s="26">
-        <v>1</v>
-      </c>
-      <c r="D28" s="30" t="s">
+      <c r="C28" s="63">
+        <v>1</v>
+      </c>
+      <c r="D28" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="E28" s="47">
-        <v>16500</v>
-      </c>
-      <c r="F28" s="46"/>
-      <c r="G28" s="46">
+      <c r="E28" s="61">
+        <v>16500</v>
+      </c>
+      <c r="F28" s="58"/>
+      <c r="G28" s="58">
         <f t="shared" si="0"/>
         <v>248908</v>
       </c>
-      <c r="H28" s="31"/>
+      <c r="H28" s="26"/>
     </row>
     <row r="29" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="17">
+      <c r="A29" s="53">
         <v>43888</v>
       </c>
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="68" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="26">
-        <v>1</v>
-      </c>
-      <c r="D29" s="30" t="s">
+      <c r="C29" s="63">
+        <v>1</v>
+      </c>
+      <c r="D29" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="49">
+      <c r="E29" s="69">
         <v>4928</v>
       </c>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46">
+      <c r="F29" s="58"/>
+      <c r="G29" s="58">
         <f t="shared" si="0"/>
         <v>253836</v>
       </c>
-      <c r="H29" s="31"/>
+      <c r="H29" s="26"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="17">
+      <c r="A30" s="53">
         <v>40141</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="29">
-        <v>1</v>
-      </c>
-      <c r="D30" s="30" t="s">
+      <c r="C30" s="64">
+        <v>1</v>
+      </c>
+      <c r="D30" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="48">
+      <c r="E30" s="65">
         <v>405.47</v>
       </c>
-      <c r="F30" s="48"/>
-      <c r="G30" s="46">
+      <c r="F30" s="65"/>
+      <c r="G30" s="58">
         <f t="shared" si="0"/>
         <v>254241.47</v>
       </c>
-      <c r="H30" s="31"/>
+      <c r="H30" s="26"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="17">
+      <c r="A31" s="53">
         <v>40141</v>
       </c>
-      <c r="B31" s="37" t="s">
+      <c r="B31" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="C31" s="19">
-        <v>1</v>
-      </c>
-      <c r="D31" s="38" t="s">
+      <c r="C31" s="55">
+        <v>1</v>
+      </c>
+      <c r="D31" s="51" t="s">
         <v>50</v>
       </c>
-      <c r="E31" s="44">
+      <c r="E31" s="56">
         <v>1680.33</v>
       </c>
-      <c r="F31" s="47"/>
-      <c r="G31" s="46">
+      <c r="F31" s="61"/>
+      <c r="G31" s="58">
         <f t="shared" si="0"/>
         <v>255921.8</v>
       </c>
-      <c r="H31" s="31"/>
+      <c r="H31" s="26"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="17"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="39" t="s">
+      <c r="A32" s="53"/>
+      <c r="B32" s="63"/>
+      <c r="C32" s="63"/>
+      <c r="D32" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="31"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="63"/>
+      <c r="G32" s="63"/>
+      <c r="H32" s="26"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="31"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="26"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H34" s="31"/>
+      <c r="H34" s="26"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E35" s="50" t="s">
+      <c r="E35" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="I35" s="40"/>
-      <c r="J35" s="31"/>
+      <c r="F35" s="44"/>
+      <c r="G35" s="44"/>
+      <c r="I35" s="34"/>
+      <c r="J35" s="26"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="31"/>
-      <c r="B36" s="31"/>
-      <c r="C36" s="41"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="41" t="s">
+      <c r="A36" s="26"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="35"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="G36" s="21"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="40"/>
-      <c r="J36" s="31"/>
+      <c r="G36" s="19"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="26"/>
     </row>
     <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
@@ -1535,15 +1606,15 @@
     <row r="4" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="55" t="s">
+      <c r="C4" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="56" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="56"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="47"/>
       <c r="I4" s="7"/>
     </row>
     <row r="5" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.35">
@@ -1560,15 +1631,15 @@
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56" t="s">
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="56"/>
+      <c r="G6" s="47"/>
     </row>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
@@ -1592,542 +1663,543 @@
       <c r="B9" s="12"/>
     </row>
     <row r="10" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="39" t="s">
+      <c r="A10" s="71"/>
+      <c r="B10" s="72"/>
+      <c r="C10" s="52"/>
+      <c r="D10" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="G10" s="53">
+      <c r="E10" s="63"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="74">
         <f>SUM('2158'!G11:G31)</f>
         <v>2767726.27</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="22" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="17">
+    <row r="11" spans="1:9" s="20" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="53">
         <v>38717</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="19">
-        <v>1</v>
-      </c>
-      <c r="D11" s="20" t="s">
+      <c r="C11" s="55">
+        <v>1</v>
+      </c>
+      <c r="D11" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="44">
+      <c r="E11" s="56">
         <v>125</v>
       </c>
-      <c r="F11" s="45"/>
-      <c r="G11" s="46">
+      <c r="F11" s="57"/>
+      <c r="G11" s="58">
         <f>(E11)</f>
         <v>125</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="22" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17">
+    <row r="12" spans="1:9" s="20" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="53">
         <v>45127</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="24">
-        <v>1</v>
-      </c>
-      <c r="D12" s="20" t="s">
+      <c r="C12" s="60">
+        <v>1</v>
+      </c>
+      <c r="D12" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="44">
+      <c r="E12" s="56">
         <v>949</v>
       </c>
-      <c r="F12" s="47"/>
-      <c r="G12" s="46">
+      <c r="F12" s="61"/>
+      <c r="G12" s="58">
         <f t="shared" ref="G12:G31" si="0">G11+E12</f>
         <v>1074</v>
       </c>
     </row>
-    <row r="13" spans="1:9" s="28" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="17">
+    <row r="13" spans="1:9" s="23" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="53">
         <v>41506</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="26">
-        <v>1</v>
-      </c>
-      <c r="D13" s="27" t="s">
+      <c r="C13" s="63">
+        <v>1</v>
+      </c>
+      <c r="D13" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="47">
+      <c r="E13" s="61">
         <v>334</v>
       </c>
-      <c r="F13" s="46"/>
-      <c r="G13" s="46">
+      <c r="F13" s="58"/>
+      <c r="G13" s="58">
         <f t="shared" si="0"/>
         <v>1408</v>
       </c>
     </row>
-    <row r="14" spans="1:9" s="28" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B14" s="29" t="s">
+    <row r="14" spans="1:9" s="23" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B14" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="29">
-        <v>1</v>
-      </c>
-      <c r="D14" s="30" t="s">
+      <c r="C14" s="64">
+        <v>1</v>
+      </c>
+      <c r="D14" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46">
+      <c r="E14" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58">
         <f t="shared" si="0"/>
         <v>17908</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B15" s="26" t="s">
+      <c r="A15" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B15" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="29">
-        <v>1</v>
-      </c>
-      <c r="D15" s="30" t="s">
+      <c r="C15" s="64">
+        <v>1</v>
+      </c>
+      <c r="D15" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="E15" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46">
+      <c r="E15" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58">
         <f t="shared" si="0"/>
         <v>34408</v>
       </c>
-      <c r="H15" s="31"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="1:9" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B16" s="29" t="s">
+      <c r="A16" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B16" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="29">
-        <v>1</v>
-      </c>
-      <c r="D16" s="30" t="s">
+      <c r="C16" s="64">
+        <v>1</v>
+      </c>
+      <c r="D16" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F16" s="46"/>
-      <c r="G16" s="46">
+      <c r="E16" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F16" s="58"/>
+      <c r="G16" s="58">
         <f t="shared" si="0"/>
         <v>50908</v>
       </c>
-      <c r="H16" s="31"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B17" s="26" t="s">
+      <c r="A17" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B17" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="26">
-        <v>1</v>
-      </c>
-      <c r="D17" s="30" t="s">
+      <c r="C17" s="63">
+        <v>1</v>
+      </c>
+      <c r="D17" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46">
+      <c r="E17" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58">
         <f t="shared" si="0"/>
         <v>67408</v>
       </c>
-      <c r="H17" s="31"/>
+      <c r="H17" s="26"/>
     </row>
     <row r="18" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B18" s="26" t="s">
+      <c r="A18" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B18" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="26">
-        <v>1</v>
-      </c>
-      <c r="D18" s="30" t="s">
+      <c r="C18" s="63">
+        <v>1</v>
+      </c>
+      <c r="D18" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46">
+      <c r="E18" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58">
         <f t="shared" si="0"/>
         <v>83908</v>
       </c>
-      <c r="H18" s="31"/>
+      <c r="H18" s="26"/>
     </row>
     <row r="19" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B19" s="32" t="s">
+      <c r="A19" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B19" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="29">
-        <v>1</v>
-      </c>
-      <c r="D19" s="30" t="s">
+      <c r="C19" s="64">
+        <v>1</v>
+      </c>
+      <c r="D19" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F19" s="46"/>
-      <c r="G19" s="46">
+      <c r="E19" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F19" s="58"/>
+      <c r="G19" s="58">
         <f t="shared" si="0"/>
         <v>100408</v>
       </c>
-      <c r="H19" s="31"/>
+      <c r="H19" s="26"/>
     </row>
     <row r="20" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B20" s="26" t="s">
+      <c r="A20" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B20" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="26">
-        <v>1</v>
-      </c>
-      <c r="D20" s="30" t="s">
+      <c r="C20" s="63">
+        <v>1</v>
+      </c>
+      <c r="D20" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46">
+      <c r="E20" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F20" s="58"/>
+      <c r="G20" s="58">
         <f t="shared" si="0"/>
         <v>116908</v>
       </c>
-      <c r="H20" s="31"/>
+      <c r="H20" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B21" s="26" t="s">
+      <c r="A21" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B21" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="26">
-        <v>1</v>
-      </c>
-      <c r="D21" s="30" t="s">
+      <c r="C21" s="63">
+        <v>1</v>
+      </c>
+      <c r="D21" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F21" s="46"/>
-      <c r="G21" s="46">
+      <c r="E21" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F21" s="58"/>
+      <c r="G21" s="58">
         <f t="shared" si="0"/>
         <v>133408</v>
       </c>
-      <c r="H21" s="31"/>
+      <c r="H21" s="26"/>
     </row>
     <row r="22" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B22" s="29" t="s">
+      <c r="A22" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B22" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="29">
-        <v>1</v>
-      </c>
-      <c r="D22" s="30" t="s">
+      <c r="C22" s="64">
+        <v>1</v>
+      </c>
+      <c r="D22" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="E22" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F22" s="46"/>
-      <c r="G22" s="46">
+      <c r="E22" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F22" s="58"/>
+      <c r="G22" s="58">
         <f t="shared" si="0"/>
         <v>149908</v>
       </c>
-      <c r="H22" s="31"/>
+      <c r="H22" s="26"/>
     </row>
     <row r="23" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B23" s="33" t="s">
+      <c r="A23" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B23" s="67" t="s">
         <v>33</v>
       </c>
-      <c r="C23" s="29">
-        <v>1</v>
-      </c>
-      <c r="D23" s="30" t="s">
+      <c r="C23" s="64">
+        <v>1</v>
+      </c>
+      <c r="D23" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="47">
-        <v>16500</v>
-      </c>
-      <c r="F23" s="45"/>
-      <c r="G23" s="46">
+      <c r="E23" s="61">
+        <v>16500</v>
+      </c>
+      <c r="F23" s="57"/>
+      <c r="G23" s="58">
         <f t="shared" si="0"/>
         <v>166408</v>
       </c>
-      <c r="H23" s="31"/>
-    </row>
-    <row r="24" spans="1:8" s="35" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B24" s="25" t="s">
+      <c r="H23" s="26"/>
+    </row>
+    <row r="24" spans="1:8" s="29" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B24" s="62" t="s">
         <v>35</v>
       </c>
-      <c r="C24" s="29">
-        <v>1</v>
-      </c>
-      <c r="D24" s="30" t="s">
+      <c r="C24" s="64">
+        <v>1</v>
+      </c>
+      <c r="D24" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F24" s="45"/>
-      <c r="G24" s="46">
+      <c r="E24" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F24" s="57"/>
+      <c r="G24" s="58">
         <f t="shared" si="0"/>
         <v>182908</v>
       </c>
-      <c r="H24" s="34"/>
-    </row>
-    <row r="25" spans="1:8" s="35" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B25" s="29" t="s">
+      <c r="H24" s="28"/>
+    </row>
+    <row r="25" spans="1:8" s="29" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B25" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="29">
-        <v>1</v>
-      </c>
-      <c r="D25" s="30" t="s">
+      <c r="C25" s="64">
+        <v>1</v>
+      </c>
+      <c r="D25" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="E25" s="47">
-        <v>16500</v>
-      </c>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46">
+      <c r="E25" s="61">
+        <v>16500</v>
+      </c>
+      <c r="F25" s="58"/>
+      <c r="G25" s="58">
         <f t="shared" si="0"/>
         <v>199408</v>
       </c>
-      <c r="H25" s="34"/>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B26" s="25" t="s">
+      <c r="A26" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B26" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="29">
-        <v>1</v>
-      </c>
-      <c r="D26" s="30" t="s">
+      <c r="C26" s="64">
+        <v>1</v>
+      </c>
+      <c r="D26" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="E26" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F26" s="46"/>
-      <c r="G26" s="46">
+      <c r="E26" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58">
         <f t="shared" si="0"/>
         <v>215908</v>
       </c>
-      <c r="H26" s="31"/>
+      <c r="H26" s="26"/>
     </row>
     <row r="27" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B27" s="25" t="s">
+      <c r="A27" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B27" s="62" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="29">
-        <v>1</v>
-      </c>
-      <c r="D27" s="30" t="s">
+      <c r="C27" s="64">
+        <v>1</v>
+      </c>
+      <c r="D27" s="50" t="s">
         <v>42</v>
       </c>
-      <c r="E27" s="47">
-        <v>16500</v>
-      </c>
-      <c r="F27" s="46"/>
-      <c r="G27" s="46">
+      <c r="E27" s="61">
+        <v>16500</v>
+      </c>
+      <c r="F27" s="58"/>
+      <c r="G27" s="58">
         <f t="shared" si="0"/>
         <v>232408</v>
       </c>
-      <c r="H27" s="31"/>
+      <c r="H27" s="26"/>
     </row>
     <row r="28" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B28" s="26" t="s">
+      <c r="A28" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B28" s="63" t="s">
         <v>43</v>
       </c>
-      <c r="C28" s="26">
-        <v>1</v>
-      </c>
-      <c r="D28" s="30" t="s">
+      <c r="C28" s="63">
+        <v>1</v>
+      </c>
+      <c r="D28" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="E28" s="47">
-        <v>16500</v>
-      </c>
-      <c r="F28" s="46"/>
-      <c r="G28" s="46">
+      <c r="E28" s="61">
+        <v>16500</v>
+      </c>
+      <c r="F28" s="58"/>
+      <c r="G28" s="58">
         <f t="shared" si="0"/>
         <v>248908</v>
       </c>
-      <c r="H28" s="31"/>
+      <c r="H28" s="26"/>
     </row>
     <row r="29" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="17">
+      <c r="A29" s="53">
         <v>43888</v>
       </c>
-      <c r="B29" s="36" t="s">
+      <c r="B29" s="68" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="26">
-        <v>1</v>
-      </c>
-      <c r="D29" s="30" t="s">
+      <c r="C29" s="63">
+        <v>1</v>
+      </c>
+      <c r="D29" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="E29" s="49">
+      <c r="E29" s="69">
         <v>4928</v>
       </c>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46">
+      <c r="F29" s="58"/>
+      <c r="G29" s="58">
         <f t="shared" si="0"/>
         <v>253836</v>
       </c>
-      <c r="H29" s="31"/>
+      <c r="H29" s="26"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="17">
+      <c r="A30" s="53">
         <v>40141</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="29">
-        <v>1</v>
-      </c>
-      <c r="D30" s="30" t="s">
+      <c r="C30" s="64">
+        <v>1</v>
+      </c>
+      <c r="D30" s="50" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="48">
+      <c r="E30" s="65">
         <v>405.47</v>
       </c>
-      <c r="F30" s="48"/>
-      <c r="G30" s="46">
+      <c r="F30" s="65"/>
+      <c r="G30" s="58">
         <f t="shared" si="0"/>
         <v>254241.47</v>
       </c>
-      <c r="H30" s="31"/>
+      <c r="H30" s="26"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="17">
+      <c r="A31" s="53">
         <v>40141</v>
       </c>
-      <c r="B31" s="37" t="s">
+      <c r="B31" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="C31" s="19">
-        <v>1</v>
-      </c>
-      <c r="D31" s="38" t="s">
+      <c r="C31" s="55">
+        <v>1</v>
+      </c>
+      <c r="D31" s="51" t="s">
         <v>50</v>
       </c>
-      <c r="E31" s="44">
+      <c r="E31" s="56">
         <v>1680.33</v>
       </c>
-      <c r="F31" s="47"/>
-      <c r="G31" s="46">
+      <c r="F31" s="61"/>
+      <c r="G31" s="58">
         <f t="shared" si="0"/>
         <v>255921.8</v>
       </c>
-      <c r="H31" s="31"/>
+      <c r="H31" s="26"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="17"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="39" t="s">
+      <c r="A32" s="53"/>
+      <c r="B32" s="63"/>
+      <c r="C32" s="63"/>
+      <c r="D32" s="52" t="s">
         <v>51</v>
       </c>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="31"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="63"/>
+      <c r="G32" s="63"/>
+      <c r="H32" s="26"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="31"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="26"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H34" s="31"/>
+      <c r="H34" s="26"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E35" s="50" t="s">
+      <c r="E35" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="I35" s="40"/>
-      <c r="J35" s="31"/>
+      <c r="F35" s="44"/>
+      <c r="G35" s="44"/>
+      <c r="I35" s="34"/>
+      <c r="J35" s="26"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="31"/>
-      <c r="B36" s="31"/>
-      <c r="C36" s="41"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="41" t="s">
+      <c r="A36" s="26"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="35"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="G36" s="21"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="40"/>
-      <c r="J36" s="31"/>
+      <c r="G36" s="19"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="26"/>
     </row>
     <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
@@ -2254,15 +2326,15 @@
     <row r="4" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5"/>
       <c r="B4" s="6"/>
-      <c r="C4" s="55" t="s">
+      <c r="C4" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="56" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="56"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="G4" s="47"/>
       <c r="I4" s="7"/>
     </row>
     <row r="5" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.35">
@@ -2279,15 +2351,15 @@
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="6"/>
-      <c r="C6" s="56" t="s">
+      <c r="C6" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56" t="s">
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="56"/>
+      <c r="G6" s="47"/>
     </row>
     <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
@@ -2311,415 +2383,416 @@
       <c r="B9" s="12"/>
     </row>
     <row r="10" spans="1:9" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="39" t="s">
+      <c r="A10" s="71"/>
+      <c r="B10" s="72"/>
+      <c r="C10" s="52"/>
+      <c r="D10" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="G10" s="54">
+      <c r="E10" s="63"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="75">
         <f>SUM('2158 (2)'!G10:G31)</f>
         <v>5535452.5399999991</v>
       </c>
     </row>
-    <row r="11" spans="1:9" s="22" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="17">
+    <row r="11" spans="1:9" s="20" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="53">
         <v>38717</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="19">
-        <v>1</v>
-      </c>
-      <c r="D11" s="20" t="s">
+      <c r="C11" s="55">
+        <v>1</v>
+      </c>
+      <c r="D11" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="44">
+      <c r="E11" s="56">
         <v>125</v>
       </c>
-      <c r="F11" s="45"/>
-      <c r="G11" s="46">
+      <c r="F11" s="57"/>
+      <c r="G11" s="58">
         <f>(E11)</f>
         <v>125</v>
       </c>
     </row>
-    <row r="12" spans="1:9" s="22" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17">
+    <row r="12" spans="1:9" s="20" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="53">
         <v>45127</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="59" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="24">
-        <v>1</v>
-      </c>
-      <c r="D12" s="20" t="s">
+      <c r="C12" s="60">
+        <v>1</v>
+      </c>
+      <c r="D12" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="44">
+      <c r="E12" s="56">
         <v>949</v>
       </c>
-      <c r="F12" s="47"/>
-      <c r="G12" s="46">
+      <c r="F12" s="61"/>
+      <c r="G12" s="58">
         <f t="shared" ref="G12:G21" si="0">G11+E12</f>
         <v>1074</v>
       </c>
     </row>
-    <row r="13" spans="1:9" s="28" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="17">
+    <row r="13" spans="1:9" s="23" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="53">
         <v>41506</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="62" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="26">
-        <v>1</v>
-      </c>
-      <c r="D13" s="27" t="s">
+      <c r="C13" s="63">
+        <v>1</v>
+      </c>
+      <c r="D13" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="47">
+      <c r="E13" s="61">
         <v>334</v>
       </c>
-      <c r="F13" s="46"/>
-      <c r="G13" s="46">
+      <c r="F13" s="58"/>
+      <c r="G13" s="58">
         <f t="shared" si="0"/>
         <v>1408</v>
       </c>
     </row>
-    <row r="14" spans="1:9" s="28" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B14" s="29" t="s">
+    <row r="14" spans="1:9" s="23" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B14" s="64" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="29">
-        <v>1</v>
-      </c>
-      <c r="D14" s="30" t="s">
+      <c r="C14" s="64">
+        <v>1</v>
+      </c>
+      <c r="D14" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46">
+      <c r="E14" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F14" s="58"/>
+      <c r="G14" s="58">
         <f t="shared" si="0"/>
         <v>17908</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B15" s="26" t="s">
+      <c r="A15" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B15" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="29">
-        <v>1</v>
-      </c>
-      <c r="D15" s="30" t="s">
+      <c r="C15" s="64">
+        <v>1</v>
+      </c>
+      <c r="D15" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="E15" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F15" s="46"/>
-      <c r="G15" s="46">
+      <c r="E15" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F15" s="58"/>
+      <c r="G15" s="58">
         <f t="shared" si="0"/>
         <v>34408</v>
       </c>
-      <c r="H15" s="31"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="1:9" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B16" s="29" t="s">
+      <c r="A16" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B16" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="29">
-        <v>1</v>
-      </c>
-      <c r="D16" s="30" t="s">
+      <c r="C16" s="64">
+        <v>1</v>
+      </c>
+      <c r="D16" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="E16" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F16" s="46"/>
-      <c r="G16" s="46">
+      <c r="E16" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F16" s="58"/>
+      <c r="G16" s="58">
         <f t="shared" si="0"/>
         <v>50908</v>
       </c>
-      <c r="H16" s="31"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B17" s="26" t="s">
+      <c r="A17" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B17" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="26">
-        <v>1</v>
-      </c>
-      <c r="D17" s="30" t="s">
+      <c r="C17" s="63">
+        <v>1</v>
+      </c>
+      <c r="D17" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F17" s="46"/>
-      <c r="G17" s="46">
+      <c r="E17" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F17" s="58"/>
+      <c r="G17" s="58">
         <f t="shared" si="0"/>
         <v>67408</v>
       </c>
-      <c r="H17" s="31"/>
+      <c r="H17" s="26"/>
     </row>
     <row r="18" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B18" s="26" t="s">
+      <c r="A18" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B18" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="26">
-        <v>1</v>
-      </c>
-      <c r="D18" s="30" t="s">
+      <c r="C18" s="63">
+        <v>1</v>
+      </c>
+      <c r="D18" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="E18" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F18" s="46"/>
-      <c r="G18" s="46">
+      <c r="E18" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F18" s="58"/>
+      <c r="G18" s="58">
         <f t="shared" si="0"/>
         <v>83908</v>
       </c>
-      <c r="H18" s="31"/>
+      <c r="H18" s="26"/>
     </row>
     <row r="19" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B19" s="32" t="s">
+      <c r="A19" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B19" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="29">
-        <v>1</v>
-      </c>
-      <c r="D19" s="30" t="s">
+      <c r="C19" s="64">
+        <v>1</v>
+      </c>
+      <c r="D19" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="48">
-        <v>16500</v>
-      </c>
-      <c r="F19" s="46"/>
-      <c r="G19" s="46">
+      <c r="E19" s="65">
+        <v>16500</v>
+      </c>
+      <c r="F19" s="58"/>
+      <c r="G19" s="58">
         <f t="shared" si="0"/>
         <v>100408</v>
       </c>
-      <c r="H19" s="31"/>
+      <c r="H19" s="26"/>
     </row>
     <row r="20" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B20" s="26" t="s">
+      <c r="A20" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B20" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="26">
-        <v>1</v>
-      </c>
-      <c r="D20" s="30" t="s">
+      <c r="C20" s="63">
+        <v>1</v>
+      </c>
+      <c r="D20" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46">
+      <c r="E20" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F20" s="58"/>
+      <c r="G20" s="58">
         <f t="shared" si="0"/>
         <v>116908</v>
       </c>
-      <c r="H20" s="31"/>
+      <c r="H20" s="26"/>
     </row>
     <row r="21" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17">
-        <v>41176</v>
-      </c>
-      <c r="B21" s="26" t="s">
+      <c r="A21" s="53">
+        <v>41176</v>
+      </c>
+      <c r="B21" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="26">
-        <v>1</v>
-      </c>
-      <c r="D21" s="30" t="s">
+      <c r="C21" s="63">
+        <v>1</v>
+      </c>
+      <c r="D21" s="50" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="46">
-        <v>16500</v>
-      </c>
-      <c r="F21" s="46"/>
-      <c r="G21" s="46">
+      <c r="E21" s="58">
+        <v>16500</v>
+      </c>
+      <c r="F21" s="58"/>
+      <c r="G21" s="58">
         <f t="shared" si="0"/>
         <v>133408</v>
       </c>
-      <c r="H21" s="31"/>
+      <c r="H21" s="26"/>
     </row>
     <row r="22" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="51" t="s">
+      <c r="A22" s="53"/>
+      <c r="B22" s="64"/>
+      <c r="C22" s="64"/>
+      <c r="D22" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="52">
+      <c r="E22" s="58"/>
+      <c r="F22" s="58"/>
+      <c r="G22" s="77">
         <f>SUM(G10:G21)</f>
         <v>6143323.5399999991</v>
       </c>
-      <c r="H22" s="31"/>
+      <c r="H22" s="26"/>
     </row>
     <row r="23" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="17"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="47"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="31"/>
-    </row>
-    <row r="24" spans="1:8" s="35" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="27"/>
+      <c r="C23" s="24"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="26"/>
+    </row>
+    <row r="24" spans="1:8" s="29" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="17"/>
-      <c r="B24" s="25"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="48"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="34"/>
-    </row>
-    <row r="25" spans="1:8" s="35" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="21"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="42"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="40"/>
+      <c r="H24" s="28"/>
+    </row>
+    <row r="25" spans="1:8" s="29" customFormat="1" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="17"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="30"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="34"/>
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="25"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="40"/>
+      <c r="H25" s="28"/>
     </row>
     <row r="26" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="17"/>
-      <c r="B26" s="25"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="46"/>
-      <c r="H26" s="31"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="40"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="26"/>
     </row>
     <row r="27" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="17"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="46"/>
-      <c r="G27" s="46"/>
-      <c r="H27" s="31"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="41"/>
+      <c r="F27" s="40"/>
+      <c r="G27" s="40"/>
+      <c r="H27" s="26"/>
     </row>
     <row r="28" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="17"/>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="46"/>
-      <c r="H28" s="31"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="41"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="26"/>
     </row>
     <row r="29" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="17"/>
-      <c r="B29" s="36"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="49"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46"/>
-      <c r="H29" s="31"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="43"/>
+      <c r="F29" s="40"/>
+      <c r="G29" s="40"/>
+      <c r="H29" s="26"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="17"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="48"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="31"/>
+      <c r="B30" s="24"/>
+      <c r="C30" s="24"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="42"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="40"/>
+      <c r="H30" s="26"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="17"/>
-      <c r="B31" s="37"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="44"/>
-      <c r="F31" s="47"/>
-      <c r="G31" s="46"/>
-      <c r="H31" s="31"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="41"/>
+      <c r="G31" s="40"/>
+      <c r="H31" s="26"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="17"/>
-      <c r="B32" s="26"/>
-      <c r="C32" s="26"/>
-      <c r="D32" s="39"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="31"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="26"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="31"/>
+      <c r="F33" s="34"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="26"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="57" t="s">
+      <c r="A34" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H34" s="31"/>
+      <c r="H34" s="26"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="E35" s="50" t="s">
+      <c r="E35" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="F35" s="50"/>
-      <c r="G35" s="50"/>
-      <c r="I35" s="40"/>
-      <c r="J35" s="31"/>
+      <c r="F35" s="44"/>
+      <c r="G35" s="44"/>
+      <c r="I35" s="34"/>
+      <c r="J35" s="26"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="31"/>
-      <c r="B36" s="31"/>
-      <c r="C36" s="41"/>
-      <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="41" t="s">
+      <c r="A36" s="26"/>
+      <c r="B36" s="26"/>
+      <c r="C36" s="35"/>
+      <c r="D36" s="36"/>
+      <c r="E36" s="37"/>
+      <c r="F36" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="G36" s="21"/>
-      <c r="H36" s="31"/>
-      <c r="I36" s="40"/>
-      <c r="J36" s="31"/>
+      <c r="G36" s="19"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="26"/>
     </row>
     <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.25"/>

</xml_diff>